<commit_message>
Import 2015/11 parliament (sejm)
</commit_message>
<xml_diff>
--- a/source-data/inbox/okregi_sejm_2019.xlsx
+++ b/source-data/inbox/okregi_sejm_2019.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57C6DB89-BF0A-43BE-8606-C8CE649298E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5400" yWindow="3345" windowWidth="21600" windowHeight="10815" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="okregi_sejm" sheetId="1" r:id="rId1"/>

</xml_diff>